<commit_message>
first part in multiple plot managment in train and test
</commit_message>
<xml_diff>
--- a/data/raw_data/season1/LAI_data_season1.xlsx
+++ b/data/raw_data/season1/LAI_data_season1.xlsx
@@ -1,20 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/beppe2hd/PycharmProjects/PureCircle/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/beppe2hd/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0547132-8B9F-AB49-9A2D-106B5A5C1F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4A6DE8D-E45E-0E4F-BA95-820E823ACA3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12880" yWindow="6980" windowWidth="51900" windowHeight="24360" activeTab="1" xr2:uid="{7C517B69-0235-47A6-840A-4957514BDF8E}"/>
+    <workbookView xWindow="7960" yWindow="1940" windowWidth="46360" windowHeight="23420" xr2:uid="{7C517B69-0235-47A6-840A-4957514BDF8E}"/>
   </bookViews>
   <sheets>
     <sheet name="LAI_S1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,34 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="14">
-  <si>
-    <t>DATE</t>
-  </si>
-  <si>
-    <t>LAI 1-CROPWAT Tititcaca</t>
-  </si>
-  <si>
-    <t>LAI 2 -Sensor Tiititcaca</t>
-  </si>
-  <si>
-    <t>LAI 3  - Farmer Titicaca</t>
-  </si>
-  <si>
-    <t>LAI 4  - CROPWAT ICBA</t>
-  </si>
-  <si>
-    <t>LAI   5 Sensor ICBA</t>
-  </si>
-  <si>
-    <t>LAI   6 Farmer ICBA</t>
-  </si>
-  <si>
-    <t>LAI1-CROPWAT-Tititcaca</t>
-  </si>
-  <si>
-    <t>LAI2-Sensor-Tiititcaca</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>LAI3-Farmer-Titicaca</t>
   </si>
@@ -72,10 +44,43 @@
     <t>LAI4-CROPWAT-ICBA</t>
   </si>
   <si>
+    <t>LAI5-Sensor-ICBA</t>
+  </si>
+  <si>
     <t>LAI6-Farmer-ICBA</t>
   </si>
   <si>
-    <t>LAI5-Sensor-ICBA</t>
+    <t>2025-02-07</t>
+  </si>
+  <si>
+    <t>2025-02-13</t>
+  </si>
+  <si>
+    <t>2025-02-20</t>
+  </si>
+  <si>
+    <t>2025-02-27</t>
+  </si>
+  <si>
+    <t>2025-03-06</t>
+  </si>
+  <si>
+    <t>2025-03-13</t>
+  </si>
+  <si>
+    <t>2025-03-20</t>
+  </si>
+  <si>
+    <t>2025-03-27</t>
+  </si>
+  <si>
+    <t>2025-04-03</t>
+  </si>
+  <si>
+    <t>LAI2-Sensor-Titicaca</t>
+  </si>
+  <si>
+    <t>LAI1-CROPWAT-Titicaca</t>
   </si>
   <si>
     <t>datetime</t>
@@ -85,7 +90,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -114,12 +119,6 @@
       <name val="Courier New"/>
       <family val="3"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -141,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -156,14 +155,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -211,7 +204,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>LAI 1-CROPWAT Tititcaca</c:v>
+                  <c:v>LAI1-CROPWAT-Titicaca</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -255,6 +248,12 @@
                 <c:pt idx="2">
                   <c:v>1.25</c:v>
                 </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.55</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.92</c:v>
+                </c:pt>
                 <c:pt idx="5">
                   <c:v>2.2599999999999998</c:v>
                 </c:pt>
@@ -286,7 +285,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>LAI 2 -Sensor Tiititcaca</c:v>
+                  <c:v>LAI5-Sensor-ICBA</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -322,31 +321,31 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>0.12</c:v>
+                  <c:v>0.37</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.5</c:v>
+                  <c:v>0.52</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.1599999999999999</c:v>
+                  <c:v>1.01</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.32</c:v>
+                  <c:v>1.67</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.79</c:v>
+                  <c:v>2.37</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2.21</c:v>
+                  <c:v>2.84</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2.89</c:v>
+                  <c:v>2.44</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2.6</c:v>
+                  <c:v>1.96</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2.38</c:v>
+                  <c:v>1.8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -366,9 +365,6 @@
               <c:f>LAI_S1!$I$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>LAI 3  - Farmer Titicaca</c:v>
-                </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
@@ -402,33 +398,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
-                <c:pt idx="0">
-                  <c:v>0.25</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.56000000000000005</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>1.07</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>1.5</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>2.48</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>2.63</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2.68</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>2.35</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>2.44</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -669,9 +638,6 @@
               <c:f>LAI_S1!$B$20</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>LAI 4  - CROPWAT ICBA</c:v>
-                </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
@@ -705,33 +671,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
-                <c:pt idx="0">
-                  <c:v>0.74</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.6</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>1.1200000000000001</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>1.66</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>2.29</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>2.61</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2.7</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>1.82</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>1.67</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -750,9 +689,6 @@
               <c:f>LAI_S1!$F$20</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>LAI   5 Sensor ICBA</c:v>
-                </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
@@ -786,33 +722,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
-                <c:pt idx="0">
-                  <c:v>0.37</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.52</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>1.01</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>1.67</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>2.37</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>2.84</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2.44</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>1.96</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>1.8</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -831,9 +740,6 @@
               <c:f>LAI_S1!$I$20</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>LAI   6 Farmer ICBA</c:v>
-                </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
@@ -867,33 +773,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
-                <c:pt idx="0">
-                  <c:v>0.21</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.64</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>1.17</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>1.68</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>2.44</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>2.72</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2.61</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>2.17</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>2.0099999999999998</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -2595,8 +2474,9 @@
   <cols>
     <col min="1" max="1" width="21.6640625" customWidth="1"/>
     <col min="2" max="2" width="31.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="18.1640625" customWidth="1"/>
+    <col min="3" max="3" width="30.33203125" customWidth="1"/>
+    <col min="4" max="4" width="29.83203125" customWidth="1"/>
+    <col min="5" max="5" width="48.1640625" customWidth="1"/>
     <col min="6" max="6" width="29.83203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19.83203125" customWidth="1"/>
     <col min="8" max="8" width="17.6640625" customWidth="1"/>
@@ -2605,226 +2485,254 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
       <c r="J1" s="3"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="4">
-        <v>20250207</v>
+      <c r="A2" s="6" t="s">
+        <v>4</v>
       </c>
       <c r="B2" s="4">
         <v>0.65</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="4"/>
+      <c r="C2" s="4">
+        <v>0.12</v>
+      </c>
+      <c r="D2" s="4">
+        <v>0.25</v>
+      </c>
       <c r="E2" s="4">
-        <v>20250207</v>
+        <v>0.74</v>
       </c>
       <c r="F2" s="4">
-        <v>0.12</v>
-      </c>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4">
-        <v>20250207</v>
-      </c>
-      <c r="I2" s="4">
-        <v>0.25</v>
-      </c>
+        <v>0.37</v>
+      </c>
+      <c r="G2" s="4">
+        <v>0.21</v>
+      </c>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="4">
-        <v>20250213</v>
+      <c r="A3" s="6" t="s">
+        <v>5</v>
       </c>
       <c r="B3" s="4">
         <v>0.65</v>
       </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="4"/>
+      <c r="C3" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="D3" s="4">
+        <v>0.56000000000000005</v>
+      </c>
       <c r="E3" s="4">
-        <v>20250213</v>
+        <v>0.6</v>
       </c>
       <c r="F3" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4">
-        <v>20250213</v>
-      </c>
-      <c r="I3" s="4">
-        <v>0.56000000000000005</v>
-      </c>
+        <v>0.52</v>
+      </c>
+      <c r="G3" s="4">
+        <v>0.64</v>
+      </c>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="4">
-        <v>20250220</v>
+      <c r="A4" s="6" t="s">
+        <v>6</v>
       </c>
       <c r="B4" s="4">
         <v>1.25</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="4"/>
+      <c r="C4" s="4">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="D4" s="4">
+        <v>1.07</v>
+      </c>
       <c r="E4" s="4">
-        <v>20250220</v>
+        <v>1.1200000000000001</v>
       </c>
       <c r="F4" s="4">
-        <v>1.1599999999999999</v>
-      </c>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4">
-        <v>20250220</v>
-      </c>
-      <c r="I4" s="4">
-        <v>1.07</v>
-      </c>
+        <v>1.01</v>
+      </c>
+      <c r="G4" s="4">
+        <v>1.17</v>
+      </c>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="4"/>
+      <c r="A5" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="4">
+        <v>1.55</v>
+      </c>
+      <c r="C5" s="4">
+        <v>1.32</v>
+      </c>
+      <c r="D5" s="4">
+        <v>1.5</v>
+      </c>
       <c r="E5" s="4">
-        <v>20250227</v>
+        <v>1.66</v>
       </c>
       <c r="F5" s="4">
-        <v>1.32</v>
-      </c>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4">
-        <v>20250227</v>
-      </c>
-      <c r="I5" s="4">
-        <v>1.5</v>
-      </c>
+        <v>1.67</v>
+      </c>
+      <c r="G5" s="4">
+        <v>1.68</v>
+      </c>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="4"/>
+      <c r="A6" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="4">
+        <v>1.92</v>
+      </c>
+      <c r="C6" s="4">
+        <v>1.79</v>
+      </c>
+      <c r="D6" s="4">
+        <v>2.48</v>
+      </c>
       <c r="E6" s="4">
-        <v>20250306</v>
+        <v>2.29</v>
       </c>
       <c r="F6" s="4">
-        <v>1.79</v>
-      </c>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4">
-        <v>20250306</v>
-      </c>
-      <c r="I6" s="4">
-        <v>2.48</v>
-      </c>
+        <v>2.37</v>
+      </c>
+      <c r="G6" s="4">
+        <v>2.44</v>
+      </c>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="4">
-        <v>20250313</v>
+      <c r="A7" s="6" t="s">
+        <v>9</v>
       </c>
       <c r="B7" s="4">
         <v>2.2599999999999998</v>
       </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="4"/>
+      <c r="C7" s="4">
+        <v>2.21</v>
+      </c>
+      <c r="D7" s="4">
+        <v>2.63</v>
+      </c>
       <c r="E7" s="4">
-        <v>20250313</v>
+        <v>2.61</v>
       </c>
       <c r="F7" s="4">
-        <v>2.21</v>
-      </c>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4">
-        <v>20250313</v>
-      </c>
-      <c r="I7" s="4">
-        <v>2.63</v>
-      </c>
+        <v>2.84</v>
+      </c>
+      <c r="G7" s="4">
+        <v>2.72</v>
+      </c>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="4">
-        <v>20250320</v>
+      <c r="A8" s="6" t="s">
+        <v>10</v>
       </c>
       <c r="B8" s="4">
         <v>1.88</v>
       </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="4"/>
+      <c r="C8" s="4">
+        <v>2.89</v>
+      </c>
+      <c r="D8" s="4">
+        <v>2.68</v>
+      </c>
       <c r="E8" s="4">
-        <v>20250320</v>
+        <v>2.7</v>
       </c>
       <c r="F8" s="4">
-        <v>2.89</v>
-      </c>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4">
-        <v>20250320</v>
-      </c>
-      <c r="I8" s="4">
-        <v>2.68</v>
-      </c>
+        <v>2.44</v>
+      </c>
+      <c r="G8" s="4">
+        <v>2.61</v>
+      </c>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="4">
-        <v>20250327</v>
+      <c r="A9" s="6" t="s">
+        <v>11</v>
       </c>
       <c r="B9" s="4">
         <v>1.91</v>
       </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="4"/>
+      <c r="C9" s="4">
+        <v>2.6</v>
+      </c>
+      <c r="D9" s="4">
+        <v>2.35</v>
+      </c>
       <c r="E9" s="4">
-        <v>20250327</v>
+        <v>1.82</v>
       </c>
       <c r="F9" s="4">
-        <v>2.6</v>
-      </c>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4">
-        <v>20250327</v>
-      </c>
-      <c r="I9" s="4">
-        <v>2.35</v>
-      </c>
+        <v>1.96</v>
+      </c>
+      <c r="G9" s="4">
+        <v>2.17</v>
+      </c>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="4">
-        <v>20250403</v>
+      <c r="A10" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="B10" s="4">
         <v>1.78</v>
       </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="4"/>
+      <c r="C10" s="4">
+        <v>2.38</v>
+      </c>
+      <c r="D10" s="4">
+        <v>2.44</v>
+      </c>
       <c r="E10" s="4">
-        <v>20250403</v>
+        <v>1.67</v>
       </c>
       <c r="F10" s="4">
-        <v>2.38</v>
-      </c>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4">
-        <v>20250403</v>
-      </c>
-      <c r="I10" s="4">
-        <v>2.44</v>
-      </c>
+        <v>1.8</v>
+      </c>
+      <c r="G10" s="4">
+        <v>2.0099999999999998</v>
+      </c>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="5"/>
@@ -2926,483 +2834,118 @@
       <c r="I19" s="5"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A20" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>4</v>
-      </c>
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
-      <c r="E20" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>5</v>
-      </c>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
       <c r="G20" s="2"/>
-      <c r="H20" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="I20" s="2" t="s">
-        <v>6</v>
-      </c>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A21" s="4">
-        <v>20250207</v>
-      </c>
-      <c r="B21" s="4">
-        <v>0.74</v>
-      </c>
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
       <c r="C21" s="5"/>
       <c r="D21" s="5"/>
-      <c r="E21" s="5">
-        <v>20250207</v>
-      </c>
-      <c r="F21" s="5">
-        <v>0.37</v>
-      </c>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
       <c r="G21" s="5"/>
-      <c r="H21" s="5">
-        <v>20250207</v>
-      </c>
-      <c r="I21" s="5">
-        <v>0.21</v>
-      </c>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A22" s="4">
-        <v>20250213</v>
-      </c>
-      <c r="B22" s="4">
-        <v>0.6</v>
-      </c>
+      <c r="A22" s="4"/>
+      <c r="B22" s="4"/>
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
-      <c r="E22" s="5">
-        <v>20250213</v>
-      </c>
-      <c r="F22" s="5">
-        <v>0.52</v>
-      </c>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
       <c r="G22" s="5"/>
-      <c r="H22" s="5">
-        <v>20250213</v>
-      </c>
-      <c r="I22" s="5">
-        <v>0.64</v>
-      </c>
+      <c r="H22" s="5"/>
+      <c r="I22" s="5"/>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A23" s="4">
-        <v>20250220</v>
-      </c>
-      <c r="B23" s="4">
-        <v>1.1200000000000001</v>
-      </c>
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
-      <c r="E23" s="5">
-        <v>20250220</v>
-      </c>
-      <c r="F23" s="5">
-        <v>1.01</v>
-      </c>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
       <c r="G23" s="5"/>
-      <c r="H23" s="5">
-        <v>20250220</v>
-      </c>
-      <c r="I23" s="5">
-        <v>1.17</v>
-      </c>
+      <c r="H23" s="5"/>
+      <c r="I23" s="5"/>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A24" s="4">
-        <v>20250227</v>
-      </c>
-      <c r="B24" s="4">
-        <v>1.66</v>
-      </c>
+      <c r="A24" s="4"/>
+      <c r="B24" s="4"/>
       <c r="C24" s="5"/>
       <c r="D24" s="5"/>
-      <c r="E24" s="5">
-        <v>20250227</v>
-      </c>
-      <c r="F24" s="5">
-        <v>1.67</v>
-      </c>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
       <c r="G24" s="5"/>
-      <c r="H24" s="5">
-        <v>20250227</v>
-      </c>
-      <c r="I24" s="5">
-        <v>1.68</v>
-      </c>
+      <c r="H24" s="5"/>
+      <c r="I24" s="5"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A25" s="4">
-        <v>20250306</v>
-      </c>
-      <c r="B25" s="4">
-        <v>2.29</v>
-      </c>
+      <c r="A25" s="4"/>
+      <c r="B25" s="4"/>
       <c r="C25" s="5"/>
       <c r="D25" s="5"/>
-      <c r="E25" s="5">
-        <v>20250306</v>
-      </c>
-      <c r="F25" s="5">
-        <v>2.37</v>
-      </c>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
       <c r="G25" s="5"/>
-      <c r="H25" s="5">
-        <v>20250306</v>
-      </c>
-      <c r="I25" s="5">
-        <v>2.44</v>
-      </c>
+      <c r="H25" s="5"/>
+      <c r="I25" s="5"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A26" s="4">
-        <v>20250313</v>
-      </c>
-      <c r="B26" s="4">
-        <v>2.61</v>
-      </c>
+      <c r="A26" s="4"/>
+      <c r="B26" s="4"/>
       <c r="C26" s="5"/>
       <c r="D26" s="5"/>
-      <c r="E26" s="5">
-        <v>20250313</v>
-      </c>
-      <c r="F26" s="5">
-        <v>2.84</v>
-      </c>
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
       <c r="G26" s="5"/>
-      <c r="H26" s="5">
-        <v>20250313</v>
-      </c>
-      <c r="I26" s="5">
-        <v>2.72</v>
-      </c>
+      <c r="H26" s="5"/>
+      <c r="I26" s="5"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A27" s="4">
-        <v>20250320</v>
-      </c>
-      <c r="B27" s="4">
-        <v>2.7</v>
-      </c>
+      <c r="A27" s="4"/>
+      <c r="B27" s="4"/>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
-      <c r="E27" s="5">
-        <v>20250320</v>
-      </c>
-      <c r="F27" s="5">
-        <v>2.44</v>
-      </c>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
       <c r="G27" s="5"/>
-      <c r="H27" s="5">
-        <v>20250320</v>
-      </c>
-      <c r="I27" s="5">
-        <v>2.61</v>
-      </c>
+      <c r="H27" s="5"/>
+      <c r="I27" s="5"/>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A28" s="4">
-        <v>20250327</v>
-      </c>
-      <c r="B28" s="4">
-        <v>1.82</v>
-      </c>
+      <c r="A28" s="4"/>
+      <c r="B28" s="4"/>
       <c r="C28" s="5"/>
       <c r="D28" s="5"/>
-      <c r="E28" s="5">
-        <v>20250327</v>
-      </c>
-      <c r="F28" s="5">
-        <v>1.96</v>
-      </c>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
       <c r="G28" s="5"/>
-      <c r="H28" s="5">
-        <v>20250327</v>
-      </c>
-      <c r="I28" s="5">
-        <v>2.17</v>
-      </c>
+      <c r="H28" s="5"/>
+      <c r="I28" s="5"/>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A29" s="4">
-        <v>20250403</v>
-      </c>
-      <c r="B29" s="4">
-        <v>1.67</v>
-      </c>
+      <c r="A29" s="4"/>
+      <c r="B29" s="4"/>
       <c r="C29" s="5"/>
       <c r="D29" s="5"/>
-      <c r="E29" s="5">
-        <v>20250403</v>
-      </c>
-      <c r="F29" s="5">
-        <v>1.8</v>
-      </c>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
       <c r="G29" s="5"/>
-      <c r="H29" s="5">
-        <v>20250403</v>
-      </c>
-      <c r="I29" s="5">
-        <v>2.0099999999999998</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0DA6A21-36A5-2342-86E4-3D1CDD143A47}">
-  <dimension ref="A1:G10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="17.83203125" customWidth="1"/>
-    <col min="2" max="2" width="27.5" customWidth="1"/>
-    <col min="3" max="3" width="28.1640625" customWidth="1"/>
-    <col min="4" max="4" width="32.5" customWidth="1"/>
-    <col min="5" max="5" width="26" customWidth="1"/>
-    <col min="6" max="6" width="19.6640625" customWidth="1"/>
-    <col min="7" max="7" width="25.1640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="6">
-        <v>45695</v>
-      </c>
-      <c r="B2" s="4">
-        <v>0.65</v>
-      </c>
-      <c r="C2" s="4">
-        <v>0.12</v>
-      </c>
-      <c r="D2" s="4">
-        <v>0.25</v>
-      </c>
-      <c r="E2" s="4">
-        <v>0.74</v>
-      </c>
-      <c r="F2" s="5">
-        <v>0.37</v>
-      </c>
-      <c r="G2" s="5">
-        <v>0.21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="6">
-        <v>45701</v>
-      </c>
-      <c r="B3" s="4">
-        <v>0.65</v>
-      </c>
-      <c r="C3" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="D3" s="4">
-        <v>0.56000000000000005</v>
-      </c>
-      <c r="E3" s="4">
-        <v>0.6</v>
-      </c>
-      <c r="F3" s="5">
-        <v>0.52</v>
-      </c>
-      <c r="G3" s="5">
-        <v>0.64</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="6">
-        <v>45708</v>
-      </c>
-      <c r="B4" s="4">
-        <v>1.25</v>
-      </c>
-      <c r="C4" s="4">
-        <v>1.1599999999999999</v>
-      </c>
-      <c r="D4" s="4">
-        <v>1.07</v>
-      </c>
-      <c r="E4" s="4">
-        <v>1.1200000000000001</v>
-      </c>
-      <c r="F4" s="5">
-        <v>1.01</v>
-      </c>
-      <c r="G4" s="5">
-        <v>1.17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="6">
-        <v>45715</v>
-      </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="4">
-        <v>1.32</v>
-      </c>
-      <c r="D5" s="4">
-        <v>1.5</v>
-      </c>
-      <c r="E5" s="4">
-        <v>1.66</v>
-      </c>
-      <c r="F5" s="5">
-        <v>1.67</v>
-      </c>
-      <c r="G5" s="5">
-        <v>1.68</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="6">
-        <v>45722</v>
-      </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="4">
-        <v>1.79</v>
-      </c>
-      <c r="D6" s="4">
-        <v>2.48</v>
-      </c>
-      <c r="E6" s="4">
-        <v>2.29</v>
-      </c>
-      <c r="F6" s="5">
-        <v>2.37</v>
-      </c>
-      <c r="G6" s="5">
-        <v>2.44</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="6">
-        <v>45729</v>
-      </c>
-      <c r="B7" s="4">
-        <v>2.2599999999999998</v>
-      </c>
-      <c r="C7" s="4">
-        <v>2.21</v>
-      </c>
-      <c r="D7" s="4">
-        <v>2.63</v>
-      </c>
-      <c r="E7" s="4">
-        <v>2.61</v>
-      </c>
-      <c r="F7" s="5">
-        <v>2.84</v>
-      </c>
-      <c r="G7" s="5">
-        <v>2.72</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="6">
-        <v>45736</v>
-      </c>
-      <c r="B8" s="4">
-        <v>1.88</v>
-      </c>
-      <c r="C8" s="4">
-        <v>2.89</v>
-      </c>
-      <c r="D8" s="4">
-        <v>2.68</v>
-      </c>
-      <c r="E8" s="4">
-        <v>2.7</v>
-      </c>
-      <c r="F8" s="5">
-        <v>2.44</v>
-      </c>
-      <c r="G8" s="5">
-        <v>2.61</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="6">
-        <v>45743</v>
-      </c>
-      <c r="B9" s="4">
-        <v>1.91</v>
-      </c>
-      <c r="C9" s="4">
-        <v>2.6</v>
-      </c>
-      <c r="D9" s="4">
-        <v>2.35</v>
-      </c>
-      <c r="E9" s="4">
-        <v>1.82</v>
-      </c>
-      <c r="F9" s="5">
-        <v>1.96</v>
-      </c>
-      <c r="G9" s="5">
-        <v>2.17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" s="6">
-        <v>45750</v>
-      </c>
-      <c r="B10" s="4">
-        <v>1.78</v>
-      </c>
-      <c r="C10" s="4">
-        <v>2.38</v>
-      </c>
-      <c r="D10" s="4">
-        <v>2.44</v>
-      </c>
-      <c r="E10" s="4">
-        <v>1.67</v>
-      </c>
-      <c r="F10" s="5">
-        <v>1.8</v>
-      </c>
-      <c r="G10" s="5">
-        <v>2.0099999999999998</v>
-      </c>
+      <c r="H29" s="5"/>
+      <c r="I29" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>